<commit_message>
W16 sales: Icedream (1,790) + Ma'ayan (12,123) + Biscotti (752) + stock + agent plan
</commit_message>
<xml_diff>
--- a/data/agents/agents_plan.xlsx
+++ b/data/agents/agents_plan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Users\עדן\דוחות שבועיים\גלידת טורבו (שבועי)\יעדי סוכנים\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\HASH-SRV\hash\Users\עדן\דוחות שבועיים\גלידת טורבו (שבועי)\יעדי סוכנים\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD9A959C-FAF4-40DB-A649-A7A3389AB105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BB17458-829D-47DC-A341-312C9AB299EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D9AFDB51-D7B9-4E57-9B64-4EC694206259}"/>
   </bookViews>
@@ -210,7 +210,7 @@
     <t>ללא מה שמסומן באדום</t>
   </si>
   <si>
-    <t>11.04.2026</t>
+    <t>18.04.2026</t>
   </si>
 </sst>
 </file>
@@ -846,7 +846,7 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -873,13 +873,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1291,21 +1285,21 @@
   <cols>
     <col min="1" max="1" width="9.125" style="7"/>
     <col min="2" max="2" width="10.625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="17" customWidth="1"/>
+    <col min="3" max="3" width="12" style="15" customWidth="1"/>
     <col min="4" max="4" width="23.125" style="7" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="19.25" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.375" style="17" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="15.375" style="15" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="12.875" style="7" customWidth="1"/>
     <col min="8" max="8" width="12.375" style="7" customWidth="1"/>
     <col min="9" max="16384" width="9.125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="27"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="25"/>
       <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
@@ -1316,9 +1310,9 @@
         <v>1</v>
       </c>
       <c r="G1" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="H1" s="18" t="s">
+        <v>0.4</v>
+      </c>
+      <c r="H1" s="16" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1336,7 +1330,7 @@
         <v>47</v>
       </c>
       <c r="G2" s="8">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H2" s="4"/>
     </row>
@@ -1367,513 +1361,532 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="17">
         <v>107</v>
       </c>
       <c r="D4" s="9">
         <v>116581.296875</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>100000</v>
       </c>
       <c r="F4" s="2">
         <v>2127.6595744680849</v>
       </c>
       <c r="G4" s="2">
-        <v>35882.62999999999</v>
-      </c>
-      <c r="H4" s="24">
-        <v>0.35882629999999988</v>
+        <v>44031.530000000006</v>
+      </c>
+      <c r="H4" s="22">
+        <f t="shared" ref="H4:H26" si="0">G4/E4</f>
+        <v>0.44031530000000008</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="17">
         <v>35</v>
       </c>
       <c r="D5" s="9">
         <v>112557.65625</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="9">
         <v>100000</v>
       </c>
       <c r="F5" s="2">
         <v>2127.6595744680849</v>
       </c>
       <c r="G5" s="2">
-        <v>18047.97</v>
-      </c>
-      <c r="H5" s="24">
-        <v>0.18047970000000002</v>
+        <v>33698.81</v>
+      </c>
+      <c r="H5" s="22">
+        <f>G5/E5</f>
+        <v>0.33698809999999996</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="17">
         <v>27</v>
       </c>
       <c r="D6" s="9">
         <v>62490.90625</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <v>70000</v>
       </c>
       <c r="F6" s="2">
         <v>1489.3617021276596</v>
       </c>
       <c r="G6" s="2">
-        <v>15792.090000000002</v>
-      </c>
-      <c r="H6" s="24">
-        <v>0.22560128571428575</v>
+        <v>31160.18</v>
+      </c>
+      <c r="H6" s="22">
+        <f t="shared" si="0"/>
+        <v>0.44514542857142858</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="17">
         <v>49</v>
       </c>
       <c r="D7" s="9">
         <v>46806.125</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="9">
         <v>50000</v>
       </c>
       <c r="F7" s="2">
         <v>1063.8297872340424</v>
       </c>
       <c r="G7" s="2">
-        <v>7038.5900000000047</v>
-      </c>
-      <c r="H7" s="24">
-        <v>0.14077180000000009</v>
+        <v>11615.160000000002</v>
+      </c>
+      <c r="H7" s="22">
+        <f t="shared" si="0"/>
+        <v>0.23230320000000004</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="17">
         <v>70</v>
       </c>
       <c r="D8" s="9">
         <v>42661.3125</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="9">
         <v>50000</v>
       </c>
       <c r="F8" s="2">
         <v>1063.8297872340424</v>
       </c>
       <c r="G8" s="2">
-        <v>25689.949999999993</v>
-      </c>
-      <c r="H8" s="24">
-        <v>0.51379899999999989</v>
+        <v>31704.089999999982</v>
+      </c>
+      <c r="H8" s="22">
+        <f t="shared" si="0"/>
+        <v>0.63408179999999958</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="17">
         <v>50</v>
       </c>
       <c r="D9" s="9">
         <v>39007.796875</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="9">
         <v>45000</v>
       </c>
       <c r="F9" s="2">
         <v>957.44680851063833</v>
       </c>
       <c r="G9" s="2">
-        <v>9446.610000000006</v>
-      </c>
-      <c r="H9" s="24">
-        <v>0.20992466666666679</v>
+        <v>13253.320000000007</v>
+      </c>
+      <c r="H9" s="22">
+        <f t="shared" si="0"/>
+        <v>0.2945182222222224</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="17">
         <v>30</v>
       </c>
       <c r="D10" s="9">
         <v>38382.109375</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="9">
         <v>45000</v>
       </c>
       <c r="F10" s="2">
         <v>957.44680851063833</v>
       </c>
       <c r="G10" s="2">
-        <v>5484.550000000002</v>
-      </c>
-      <c r="H10" s="24">
-        <v>0.12187888888888894</v>
+        <v>13465.600000000002</v>
+      </c>
+      <c r="H10" s="22">
+        <f t="shared" si="0"/>
+        <v>0.29923555555555559</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="17">
         <v>41</v>
       </c>
       <c r="D11" s="9">
         <v>36472</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="9">
         <v>45000</v>
       </c>
       <c r="F11" s="2">
         <v>957.44680851063833</v>
       </c>
       <c r="G11" s="2">
-        <v>9436.67</v>
-      </c>
-      <c r="H11" s="24">
-        <v>0.20970377777777777</v>
+        <v>11692.220000000003</v>
+      </c>
+      <c r="H11" s="22">
+        <f t="shared" si="0"/>
+        <v>0.25982711111111118</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="17">
         <v>44</v>
       </c>
       <c r="D12" s="9">
         <v>23593.265625</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="9">
         <v>30000</v>
       </c>
       <c r="F12" s="2">
         <v>638.29787234042556</v>
       </c>
       <c r="G12" s="2">
-        <v>9023.9200000000019</v>
-      </c>
-      <c r="H12" s="24">
-        <v>0.30079733333333342</v>
+        <v>13536.650000000007</v>
+      </c>
+      <c r="H12" s="22">
+        <f t="shared" si="0"/>
+        <v>0.45122166666666691</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="17">
         <v>37</v>
       </c>
       <c r="D13" s="9">
         <v>23247.375</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="9">
         <v>30000</v>
       </c>
       <c r="F13" s="2">
         <v>638.29787234042556</v>
       </c>
       <c r="G13" s="2">
-        <v>1832.3300000000002</v>
-      </c>
-      <c r="H13" s="24">
-        <v>6.1077666666666669E-2</v>
+        <v>4229.8500000000013</v>
+      </c>
+      <c r="H13" s="22">
+        <f t="shared" si="0"/>
+        <v>0.14099500000000004</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="17">
         <v>40</v>
       </c>
       <c r="D14" s="9">
         <v>20507.421875</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="9">
         <v>30000</v>
       </c>
       <c r="F14" s="2">
         <v>638.29787234042556</v>
       </c>
       <c r="G14" s="2">
-        <v>4011.6299999999997</v>
-      </c>
-      <c r="H14" s="24">
-        <v>0.13372099999999998</v>
+        <v>5562.7699999999986</v>
+      </c>
+      <c r="H14" s="22">
+        <f t="shared" si="0"/>
+        <v>0.18542566666666663</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="17">
         <v>29</v>
       </c>
       <c r="D15" s="9">
         <v>20299.59375</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="9">
         <v>30000</v>
       </c>
       <c r="F15" s="2">
         <v>638.29787234042556</v>
       </c>
       <c r="G15" s="2">
-        <v>1832.58</v>
-      </c>
-      <c r="H15" s="24">
-        <v>6.1085999999999994E-2</v>
+        <v>4243.66</v>
+      </c>
+      <c r="H15" s="22">
+        <f t="shared" si="0"/>
+        <v>0.14145533333333332</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="17">
         <v>28</v>
       </c>
       <c r="D16" s="9">
         <v>19950.765625</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="9">
         <v>30000</v>
       </c>
       <c r="F16" s="2">
         <v>638.29787234042556</v>
       </c>
       <c r="G16" s="2">
-        <v>3799.0100000000007</v>
-      </c>
-      <c r="H16" s="24">
-        <v>0.1266336666666667</v>
+        <v>5632.25</v>
+      </c>
+      <c r="H16" s="22">
+        <f t="shared" si="0"/>
+        <v>0.18774166666666667</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="17">
         <v>28</v>
       </c>
       <c r="D17" s="9">
         <v>17230.640625</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="9">
         <v>20000</v>
       </c>
       <c r="F17" s="2">
         <v>425.531914893617</v>
       </c>
       <c r="G17" s="2">
-        <v>4876.3100000000013</v>
-      </c>
-      <c r="H17" s="24">
-        <v>0.24381550000000007</v>
+        <v>8091.9600000000028</v>
+      </c>
+      <c r="H17" s="22">
+        <f t="shared" si="0"/>
+        <v>0.40459800000000012</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="17">
         <v>19</v>
       </c>
       <c r="D18" s="9">
         <v>10901.796875</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="9">
         <v>25000</v>
       </c>
       <c r="F18" s="2">
         <v>531.91489361702122</v>
       </c>
       <c r="G18" s="2">
-        <v>3039.2700000000004</v>
-      </c>
-      <c r="H18" s="24">
-        <v>0.12157080000000002</v>
+        <v>4872.2700000000023</v>
+      </c>
+      <c r="H18" s="22">
+        <f t="shared" si="0"/>
+        <v>0.19489080000000009</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="19">
+      <c r="C19" s="17">
         <v>30</v>
       </c>
       <c r="D19" s="9">
         <v>10162.28125</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="9">
         <v>20000</v>
       </c>
       <c r="F19" s="2">
         <v>425.531914893617</v>
       </c>
       <c r="G19" s="2">
-        <v>2820.3899999999994</v>
-      </c>
-      <c r="H19" s="24">
-        <v>0.14101949999999996</v>
+        <v>2961.4699999999993</v>
+      </c>
+      <c r="H19" s="22">
+        <f t="shared" si="0"/>
+        <v>0.14807349999999997</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="17">
         <v>12</v>
       </c>
       <c r="D20" s="9">
         <v>8836</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="9">
         <v>20000</v>
       </c>
       <c r="F20" s="2">
         <v>425.531914893617</v>
       </c>
       <c r="G20" s="2">
-        <v>2679.22</v>
-      </c>
-      <c r="H20" s="24">
-        <v>0.133961</v>
+        <v>3384.0199999999995</v>
+      </c>
+      <c r="H20" s="22">
+        <f t="shared" si="0"/>
+        <v>0.16920099999999996</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="17">
         <v>16</v>
       </c>
       <c r="D21" s="9">
         <v>4744.796875</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="9">
         <v>20000</v>
       </c>
       <c r="F21" s="2">
         <v>425.531914893617</v>
       </c>
       <c r="G21" s="2">
-        <v>1128.06</v>
-      </c>
-      <c r="H21" s="24">
-        <v>5.6402999999999995E-2</v>
+        <v>4063.4199999999992</v>
+      </c>
+      <c r="H21" s="22">
+        <f t="shared" si="0"/>
+        <v>0.20317099999999996</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="17">
         <v>12</v>
       </c>
       <c r="D22" s="9">
         <v>4356.3125</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="9">
         <v>20000</v>
       </c>
       <c r="F22" s="2">
         <v>425.531914893617</v>
       </c>
       <c r="G22" s="2">
-        <v>1512.7099999999998</v>
-      </c>
-      <c r="H22" s="24">
-        <v>7.5635499999999994E-2</v>
+        <v>3730.130000000001</v>
+      </c>
+      <c r="H22" s="22">
+        <f t="shared" si="0"/>
+        <v>0.18650650000000005</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="18">
         <v>4</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <v>4147.015625</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="10">
         <v>5000</v>
       </c>
       <c r="F23" s="3">
@@ -1882,24 +1895,25 @@
       <c r="G23" s="2">
         <v>987.28000000000009</v>
       </c>
-      <c r="H23" s="24">
+      <c r="H23" s="22">
+        <f t="shared" si="0"/>
         <v>0.19745600000000002</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="18">
         <v>9</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="10">
         <v>2549.015625</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="10">
         <v>5000</v>
       </c>
       <c r="F24" s="3">
@@ -1908,50 +1922,52 @@
       <c r="G24" s="2">
         <v>0</v>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="22">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="18">
         <v>3</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <v>1077.328125</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="10">
         <v>5000</v>
       </c>
       <c r="F25" s="3">
         <v>106.38297872340425</v>
       </c>
       <c r="G25" s="2">
-        <v>423.15000000000003</v>
-      </c>
-      <c r="H25" s="24">
-        <v>8.4630000000000011E-2</v>
+        <v>705.11</v>
+      </c>
+      <c r="H25" s="22">
+        <f t="shared" si="0"/>
+        <v>0.14102200000000001</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="18">
         <v>1</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="10">
         <v>62.421875</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="10">
         <v>5000</v>
       </c>
       <c r="F26" s="3">
@@ -1960,7 +1976,8 @@
       <c r="G26" s="2">
         <v>0</v>
       </c>
-      <c r="H26" s="24">
+      <c r="H26" s="22">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1974,32 +1991,33 @@
       <c r="C27" s="1">
         <v>721</v>
       </c>
-      <c r="D27" s="13">
+      <c r="D27" s="11">
         <v>666625.234375</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27" s="21">
         <v>780000</v>
       </c>
-      <c r="F27" s="13">
+      <c r="F27" s="11">
         <v>17021.276595744672</v>
       </c>
-      <c r="G27" s="23">
-        <v>164784.91999999998</v>
-      </c>
-      <c r="H27" s="14">
-        <v>0.21126271794871793</v>
+      <c r="G27" s="21">
+        <f>SUM(G4:G26)</f>
+        <v>252621.74999999994</v>
+      </c>
+      <c r="H27" s="12">
+        <v>0.32</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="16" t="s">
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14" t="s">
         <v>57</v>
       </c>
       <c r="F28" s="2"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Update agent plan to 26 Apr version (data date 25/4)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/agents/agents_plan.xlsx
+++ b/data/agents/agents_plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\HASH-SRV\hash\Users\עדן\דוחות שבועיים\גלידת טורבו (שבועי)\יעדי סוכנים\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BB17458-829D-47DC-A341-312C9AB299EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DD7CEBA-E762-477F-8ACB-AE291D7FE9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D9AFDB51-D7B9-4E57-9B64-4EC694206259}"/>
   </bookViews>
@@ -210,7 +210,7 @@
     <t>ללא מה שמסומן באדום</t>
   </si>
   <si>
-    <t>18.04.2026</t>
+    <t>25.04.2026</t>
   </si>
 </sst>
 </file>
@@ -1310,7 +1310,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="6">
-        <v>0.4</v>
+        <v>0.51</v>
       </c>
       <c r="H1" s="16" t="s">
         <v>58</v>
@@ -1330,7 +1330,7 @@
         <v>47</v>
       </c>
       <c r="G2" s="8">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H2" s="4"/>
     </row>
@@ -1380,11 +1380,11 @@
         <v>2127.6595744680849</v>
       </c>
       <c r="G4" s="2">
-        <v>44031.530000000006</v>
+        <v>55786.630000000005</v>
       </c>
       <c r="H4" s="22">
         <f t="shared" ref="H4:H26" si="0">G4/E4</f>
-        <v>0.44031530000000008</v>
+        <v>0.55786630000000004</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1407,11 +1407,11 @@
         <v>2127.6595744680849</v>
       </c>
       <c r="G5" s="2">
-        <v>33698.81</v>
+        <v>34121.630000000005</v>
       </c>
       <c r="H5" s="22">
         <f>G5/E5</f>
-        <v>0.33698809999999996</v>
+        <v>0.34121630000000003</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1461,11 +1461,11 @@
         <v>1063.8297872340424</v>
       </c>
       <c r="G7" s="2">
-        <v>11615.160000000002</v>
+        <v>16274.820000000002</v>
       </c>
       <c r="H7" s="22">
         <f t="shared" si="0"/>
-        <v>0.23230320000000004</v>
+        <v>0.32549640000000002</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1488,11 +1488,11 @@
         <v>1063.8297872340424</v>
       </c>
       <c r="G8" s="2">
-        <v>31704.089999999982</v>
+        <v>33099.869999999988</v>
       </c>
       <c r="H8" s="22">
         <f t="shared" si="0"/>
-        <v>0.63408179999999958</v>
+        <v>0.66199739999999974</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1515,11 +1515,11 @@
         <v>957.44680851063833</v>
       </c>
       <c r="G9" s="2">
-        <v>13253.320000000007</v>
+        <v>15228.150000000011</v>
       </c>
       <c r="H9" s="22">
         <f t="shared" si="0"/>
-        <v>0.2945182222222224</v>
+        <v>0.33840333333333356</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1542,11 +1542,11 @@
         <v>957.44680851063833</v>
       </c>
       <c r="G10" s="2">
-        <v>13465.600000000002</v>
+        <v>18964.59</v>
       </c>
       <c r="H10" s="22">
         <f t="shared" si="0"/>
-        <v>0.29923555555555559</v>
+        <v>0.42143533333333333</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1569,11 +1569,11 @@
         <v>957.44680851063833</v>
       </c>
       <c r="G11" s="2">
-        <v>11692.220000000003</v>
+        <v>14794.500000000004</v>
       </c>
       <c r="H11" s="22">
         <f t="shared" si="0"/>
-        <v>0.25982711111111118</v>
+        <v>0.32876666666666676</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1596,11 +1596,11 @@
         <v>638.29787234042556</v>
       </c>
       <c r="G12" s="2">
-        <v>13536.650000000007</v>
+        <v>14664.400000000005</v>
       </c>
       <c r="H12" s="22">
         <f t="shared" si="0"/>
-        <v>0.45122166666666691</v>
+        <v>0.48881333333333349</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1623,11 +1623,11 @@
         <v>638.29787234042556</v>
       </c>
       <c r="G13" s="2">
-        <v>4229.8500000000013</v>
+        <v>6908.8800000000028</v>
       </c>
       <c r="H13" s="22">
         <f t="shared" si="0"/>
-        <v>0.14099500000000004</v>
+        <v>0.23029600000000008</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1650,11 +1650,11 @@
         <v>638.29787234042556</v>
       </c>
       <c r="G14" s="2">
-        <v>5562.7699999999986</v>
+        <v>6126.7699999999986</v>
       </c>
       <c r="H14" s="22">
         <f t="shared" si="0"/>
-        <v>0.18542566666666663</v>
+        <v>0.20422566666666661</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1677,11 +1677,11 @@
         <v>638.29787234042556</v>
       </c>
       <c r="G15" s="2">
-        <v>4243.66</v>
+        <v>4384.67</v>
       </c>
       <c r="H15" s="22">
         <f t="shared" si="0"/>
-        <v>0.14145533333333332</v>
+        <v>0.14615566666666666</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1704,11 +1704,11 @@
         <v>638.29787234042556</v>
       </c>
       <c r="G16" s="2">
-        <v>5632.25</v>
+        <v>6055.2800000000007</v>
       </c>
       <c r="H16" s="22">
         <f t="shared" si="0"/>
-        <v>0.18774166666666667</v>
+        <v>0.2018426666666667</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1731,11 +1731,11 @@
         <v>425.531914893617</v>
       </c>
       <c r="G17" s="2">
-        <v>8091.9600000000028</v>
+        <v>10389.73</v>
       </c>
       <c r="H17" s="22">
         <f t="shared" si="0"/>
-        <v>0.40459800000000012</v>
+        <v>0.51948649999999996</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1785,11 +1785,11 @@
         <v>425.531914893617</v>
       </c>
       <c r="G19" s="2">
-        <v>2961.4699999999993</v>
+        <v>2820.7899999999995</v>
       </c>
       <c r="H19" s="22">
         <f t="shared" si="0"/>
-        <v>0.14807349999999997</v>
+        <v>0.14103949999999998</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1812,11 +1812,11 @@
         <v>425.531914893617</v>
       </c>
       <c r="G20" s="2">
-        <v>3384.0199999999995</v>
+        <v>4652.619999999999</v>
       </c>
       <c r="H20" s="22">
         <f t="shared" si="0"/>
-        <v>0.16920099999999996</v>
+        <v>0.23263099999999995</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1839,11 +1839,11 @@
         <v>425.531914893617</v>
       </c>
       <c r="G21" s="2">
-        <v>4063.4199999999992</v>
+        <v>6743.1400000000021</v>
       </c>
       <c r="H21" s="22">
         <f t="shared" si="0"/>
-        <v>0.20317099999999996</v>
+        <v>0.3371570000000001</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1866,11 +1866,11 @@
         <v>425.531914893617</v>
       </c>
       <c r="G22" s="2">
-        <v>3730.130000000001</v>
+        <v>4828.6400000000003</v>
       </c>
       <c r="H22" s="22">
         <f t="shared" si="0"/>
-        <v>0.18650650000000005</v>
+        <v>0.24143200000000001</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -1920,11 +1920,11 @@
         <v>106.38297872340425</v>
       </c>
       <c r="G24" s="2">
-        <v>0</v>
+        <v>564.08000000000004</v>
       </c>
       <c r="H24" s="22">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.11281600000000001</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="G27" s="21">
         <f>SUM(G4:G26)</f>
-        <v>252621.74999999994</v>
+        <v>294134.03000000009</v>
       </c>
       <c r="H27" s="12">
         <v>0.32</v>

</xml_diff>